<commit_message>
TN1 vérifié dans Google Sheets : formule robuste aux cases effacées (=TRUE), page corrigée (ligne 3, bandeau, remise à FAUX, colonne Catégorie), deux captures d'écran
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TN1-systeme-expert-animaux.xlsx
+++ b/TN1-systeme-expert-animaux.xlsx
@@ -1281,7 +1281,7 @@
         </is>
       </c>
       <c r="G3" s="10">
-        <f>IF($F3="","",AND(IF($B3="",TRUE,VLOOKUP($B3,Faits!$A:$B,2,FALSE)),IF($C3="",TRUE,VLOOKUP($C3,Faits!$A:$B,2,FALSE)),IF($D3="",TRUE,VLOOKUP($D3,Faits!$A:$B,2,FALSE)),IF($E3="",TRUE,VLOOKUP($E3,Faits!$A:$B,2,FALSE)),NOT(VLOOKUP($F3,Faits!$A:$B,2,FALSE))))</f>
+        <f>IF($F3="","",AND(IF($B3="",TRUE,VLOOKUP($B3,Faits!$A:$B,2,FALSE)=TRUE),IF($C3="",TRUE,VLOOKUP($C3,Faits!$A:$B,2,FALSE)=TRUE),IF($D3="",TRUE,VLOOKUP($D3,Faits!$A:$B,2,FALSE)=TRUE),IF($E3="",TRUE,VLOOKUP($E3,Faits!$A:$B,2,FALSE)=TRUE),VLOOKUP($F3,Faits!$A:$B,2,FALSE)&lt;&gt;TRUE))</f>
         <v/>
       </c>
       <c r="H3" s="10">
@@ -1309,7 +1309,7 @@
         </is>
       </c>
       <c r="G4" s="10">
-        <f>IF($F4="","",AND(IF($B4="",TRUE,VLOOKUP($B4,Faits!$A:$B,2,FALSE)),IF($C4="",TRUE,VLOOKUP($C4,Faits!$A:$B,2,FALSE)),IF($D4="",TRUE,VLOOKUP($D4,Faits!$A:$B,2,FALSE)),IF($E4="",TRUE,VLOOKUP($E4,Faits!$A:$B,2,FALSE)),NOT(VLOOKUP($F4,Faits!$A:$B,2,FALSE))))</f>
+        <f>IF($F4="","",AND(IF($B4="",TRUE,VLOOKUP($B4,Faits!$A:$B,2,FALSE)=TRUE),IF($C4="",TRUE,VLOOKUP($C4,Faits!$A:$B,2,FALSE)=TRUE),IF($D4="",TRUE,VLOOKUP($D4,Faits!$A:$B,2,FALSE)=TRUE),IF($E4="",TRUE,VLOOKUP($E4,Faits!$A:$B,2,FALSE)=TRUE),VLOOKUP($F4,Faits!$A:$B,2,FALSE)&lt;&gt;TRUE))</f>
         <v/>
       </c>
       <c r="H4" s="10">
@@ -1337,7 +1337,7 @@
         </is>
       </c>
       <c r="G5" s="10">
-        <f>IF($F5="","",AND(IF($B5="",TRUE,VLOOKUP($B5,Faits!$A:$B,2,FALSE)),IF($C5="",TRUE,VLOOKUP($C5,Faits!$A:$B,2,FALSE)),IF($D5="",TRUE,VLOOKUP($D5,Faits!$A:$B,2,FALSE)),IF($E5="",TRUE,VLOOKUP($E5,Faits!$A:$B,2,FALSE)),NOT(VLOOKUP($F5,Faits!$A:$B,2,FALSE))))</f>
+        <f>IF($F5="","",AND(IF($B5="",TRUE,VLOOKUP($B5,Faits!$A:$B,2,FALSE)=TRUE),IF($C5="",TRUE,VLOOKUP($C5,Faits!$A:$B,2,FALSE)=TRUE),IF($D5="",TRUE,VLOOKUP($D5,Faits!$A:$B,2,FALSE)=TRUE),IF($E5="",TRUE,VLOOKUP($E5,Faits!$A:$B,2,FALSE)=TRUE),VLOOKUP($F5,Faits!$A:$B,2,FALSE)&lt;&gt;TRUE))</f>
         <v/>
       </c>
       <c r="H5" s="10">
@@ -1369,7 +1369,7 @@
         </is>
       </c>
       <c r="G6" s="10">
-        <f>IF($F6="","",AND(IF($B6="",TRUE,VLOOKUP($B6,Faits!$A:$B,2,FALSE)),IF($C6="",TRUE,VLOOKUP($C6,Faits!$A:$B,2,FALSE)),IF($D6="",TRUE,VLOOKUP($D6,Faits!$A:$B,2,FALSE)),IF($E6="",TRUE,VLOOKUP($E6,Faits!$A:$B,2,FALSE)),NOT(VLOOKUP($F6,Faits!$A:$B,2,FALSE))))</f>
+        <f>IF($F6="","",AND(IF($B6="",TRUE,VLOOKUP($B6,Faits!$A:$B,2,FALSE)=TRUE),IF($C6="",TRUE,VLOOKUP($C6,Faits!$A:$B,2,FALSE)=TRUE),IF($D6="",TRUE,VLOOKUP($D6,Faits!$A:$B,2,FALSE)=TRUE),IF($E6="",TRUE,VLOOKUP($E6,Faits!$A:$B,2,FALSE)=TRUE),VLOOKUP($F6,Faits!$A:$B,2,FALSE)&lt;&gt;TRUE))</f>
         <v/>
       </c>
       <c r="H6" s="10">
@@ -1405,7 +1405,7 @@
         </is>
       </c>
       <c r="G7" s="10">
-        <f>IF($F7="","",AND(IF($B7="",TRUE,VLOOKUP($B7,Faits!$A:$B,2,FALSE)),IF($C7="",TRUE,VLOOKUP($C7,Faits!$A:$B,2,FALSE)),IF($D7="",TRUE,VLOOKUP($D7,Faits!$A:$B,2,FALSE)),IF($E7="",TRUE,VLOOKUP($E7,Faits!$A:$B,2,FALSE)),NOT(VLOOKUP($F7,Faits!$A:$B,2,FALSE))))</f>
+        <f>IF($F7="","",AND(IF($B7="",TRUE,VLOOKUP($B7,Faits!$A:$B,2,FALSE)=TRUE),IF($C7="",TRUE,VLOOKUP($C7,Faits!$A:$B,2,FALSE)=TRUE),IF($D7="",TRUE,VLOOKUP($D7,Faits!$A:$B,2,FALSE)=TRUE),IF($E7="",TRUE,VLOOKUP($E7,Faits!$A:$B,2,FALSE)=TRUE),VLOOKUP($F7,Faits!$A:$B,2,FALSE)&lt;&gt;TRUE))</f>
         <v/>
       </c>
       <c r="H7" s="10">
@@ -1441,7 +1441,7 @@
         </is>
       </c>
       <c r="G8" s="10">
-        <f>IF($F8="","",AND(IF($B8="",TRUE,VLOOKUP($B8,Faits!$A:$B,2,FALSE)),IF($C8="",TRUE,VLOOKUP($C8,Faits!$A:$B,2,FALSE)),IF($D8="",TRUE,VLOOKUP($D8,Faits!$A:$B,2,FALSE)),IF($E8="",TRUE,VLOOKUP($E8,Faits!$A:$B,2,FALSE)),NOT(VLOOKUP($F8,Faits!$A:$B,2,FALSE))))</f>
+        <f>IF($F8="","",AND(IF($B8="",TRUE,VLOOKUP($B8,Faits!$A:$B,2,FALSE)=TRUE),IF($C8="",TRUE,VLOOKUP($C8,Faits!$A:$B,2,FALSE)=TRUE),IF($D8="",TRUE,VLOOKUP($D8,Faits!$A:$B,2,FALSE)=TRUE),IF($E8="",TRUE,VLOOKUP($E8,Faits!$A:$B,2,FALSE)=TRUE),VLOOKUP($F8,Faits!$A:$B,2,FALSE)&lt;&gt;TRUE))</f>
         <v/>
       </c>
       <c r="H8" s="10">
@@ -1477,7 +1477,7 @@
         </is>
       </c>
       <c r="G9" s="10">
-        <f>IF($F9="","",AND(IF($B9="",TRUE,VLOOKUP($B9,Faits!$A:$B,2,FALSE)),IF($C9="",TRUE,VLOOKUP($C9,Faits!$A:$B,2,FALSE)),IF($D9="",TRUE,VLOOKUP($D9,Faits!$A:$B,2,FALSE)),IF($E9="",TRUE,VLOOKUP($E9,Faits!$A:$B,2,FALSE)),NOT(VLOOKUP($F9,Faits!$A:$B,2,FALSE))))</f>
+        <f>IF($F9="","",AND(IF($B9="",TRUE,VLOOKUP($B9,Faits!$A:$B,2,FALSE)=TRUE),IF($C9="",TRUE,VLOOKUP($C9,Faits!$A:$B,2,FALSE)=TRUE),IF($D9="",TRUE,VLOOKUP($D9,Faits!$A:$B,2,FALSE)=TRUE),IF($E9="",TRUE,VLOOKUP($E9,Faits!$A:$B,2,FALSE)=TRUE),VLOOKUP($F9,Faits!$A:$B,2,FALSE)&lt;&gt;TRUE))</f>
         <v/>
       </c>
       <c r="H9" s="10">
@@ -1517,7 +1517,7 @@
         </is>
       </c>
       <c r="G10" s="10">
-        <f>IF($F10="","",AND(IF($B10="",TRUE,VLOOKUP($B10,Faits!$A:$B,2,FALSE)),IF($C10="",TRUE,VLOOKUP($C10,Faits!$A:$B,2,FALSE)),IF($D10="",TRUE,VLOOKUP($D10,Faits!$A:$B,2,FALSE)),IF($E10="",TRUE,VLOOKUP($E10,Faits!$A:$B,2,FALSE)),NOT(VLOOKUP($F10,Faits!$A:$B,2,FALSE))))</f>
+        <f>IF($F10="","",AND(IF($B10="",TRUE,VLOOKUP($B10,Faits!$A:$B,2,FALSE)=TRUE),IF($C10="",TRUE,VLOOKUP($C10,Faits!$A:$B,2,FALSE)=TRUE),IF($D10="",TRUE,VLOOKUP($D10,Faits!$A:$B,2,FALSE)=TRUE),IF($E10="",TRUE,VLOOKUP($E10,Faits!$A:$B,2,FALSE)=TRUE),VLOOKUP($F10,Faits!$A:$B,2,FALSE)&lt;&gt;TRUE))</f>
         <v/>
       </c>
       <c r="H10" s="10">
@@ -1553,7 +1553,7 @@
         </is>
       </c>
       <c r="G11" s="10">
-        <f>IF($F11="","",AND(IF($B11="",TRUE,VLOOKUP($B11,Faits!$A:$B,2,FALSE)),IF($C11="",TRUE,VLOOKUP($C11,Faits!$A:$B,2,FALSE)),IF($D11="",TRUE,VLOOKUP($D11,Faits!$A:$B,2,FALSE)),IF($E11="",TRUE,VLOOKUP($E11,Faits!$A:$B,2,FALSE)),NOT(VLOOKUP($F11,Faits!$A:$B,2,FALSE))))</f>
+        <f>IF($F11="","",AND(IF($B11="",TRUE,VLOOKUP($B11,Faits!$A:$B,2,FALSE)=TRUE),IF($C11="",TRUE,VLOOKUP($C11,Faits!$A:$B,2,FALSE)=TRUE),IF($D11="",TRUE,VLOOKUP($D11,Faits!$A:$B,2,FALSE)=TRUE),IF($E11="",TRUE,VLOOKUP($E11,Faits!$A:$B,2,FALSE)=TRUE),VLOOKUP($F11,Faits!$A:$B,2,FALSE)&lt;&gt;TRUE))</f>
         <v/>
       </c>
       <c r="H11" s="10">
@@ -1589,7 +1589,7 @@
         </is>
       </c>
       <c r="G12" s="10">
-        <f>IF($F12="","",AND(IF($B12="",TRUE,VLOOKUP($B12,Faits!$A:$B,2,FALSE)),IF($C12="",TRUE,VLOOKUP($C12,Faits!$A:$B,2,FALSE)),IF($D12="",TRUE,VLOOKUP($D12,Faits!$A:$B,2,FALSE)),IF($E12="",TRUE,VLOOKUP($E12,Faits!$A:$B,2,FALSE)),NOT(VLOOKUP($F12,Faits!$A:$B,2,FALSE))))</f>
+        <f>IF($F12="","",AND(IF($B12="",TRUE,VLOOKUP($B12,Faits!$A:$B,2,FALSE)=TRUE),IF($C12="",TRUE,VLOOKUP($C12,Faits!$A:$B,2,FALSE)=TRUE),IF($D12="",TRUE,VLOOKUP($D12,Faits!$A:$B,2,FALSE)=TRUE),IF($E12="",TRUE,VLOOKUP($E12,Faits!$A:$B,2,FALSE)=TRUE),VLOOKUP($F12,Faits!$A:$B,2,FALSE)&lt;&gt;TRUE))</f>
         <v/>
       </c>
       <c r="H12" s="10">
@@ -1629,7 +1629,7 @@
         </is>
       </c>
       <c r="G13" s="10">
-        <f>IF($F13="","",AND(IF($B13="",TRUE,VLOOKUP($B13,Faits!$A:$B,2,FALSE)),IF($C13="",TRUE,VLOOKUP($C13,Faits!$A:$B,2,FALSE)),IF($D13="",TRUE,VLOOKUP($D13,Faits!$A:$B,2,FALSE)),IF($E13="",TRUE,VLOOKUP($E13,Faits!$A:$B,2,FALSE)),NOT(VLOOKUP($F13,Faits!$A:$B,2,FALSE))))</f>
+        <f>IF($F13="","",AND(IF($B13="",TRUE,VLOOKUP($B13,Faits!$A:$B,2,FALSE)=TRUE),IF($C13="",TRUE,VLOOKUP($C13,Faits!$A:$B,2,FALSE)=TRUE),IF($D13="",TRUE,VLOOKUP($D13,Faits!$A:$B,2,FALSE)=TRUE),IF($E13="",TRUE,VLOOKUP($E13,Faits!$A:$B,2,FALSE)=TRUE),VLOOKUP($F13,Faits!$A:$B,2,FALSE)&lt;&gt;TRUE))</f>
         <v/>
       </c>
       <c r="H13" s="10">
@@ -1645,7 +1645,7 @@
       <c r="E14" s="2" t="n"/>
       <c r="F14" s="2" t="n"/>
       <c r="G14" s="10">
-        <f>IF($F14="","",AND(IF($B14="",TRUE,VLOOKUP($B14,Faits!$A:$B,2,FALSE)),IF($C14="",TRUE,VLOOKUP($C14,Faits!$A:$B,2,FALSE)),IF($D14="",TRUE,VLOOKUP($D14,Faits!$A:$B,2,FALSE)),IF($E14="",TRUE,VLOOKUP($E14,Faits!$A:$B,2,FALSE)),NOT(VLOOKUP($F14,Faits!$A:$B,2,FALSE))))</f>
+        <f>IF($F14="","",AND(IF($B14="",TRUE,VLOOKUP($B14,Faits!$A:$B,2,FALSE)=TRUE),IF($C14="",TRUE,VLOOKUP($C14,Faits!$A:$B,2,FALSE)=TRUE),IF($D14="",TRUE,VLOOKUP($D14,Faits!$A:$B,2,FALSE)=TRUE),IF($E14="",TRUE,VLOOKUP($E14,Faits!$A:$B,2,FALSE)=TRUE),VLOOKUP($F14,Faits!$A:$B,2,FALSE)&lt;&gt;TRUE))</f>
         <v/>
       </c>
       <c r="H14" s="10">
@@ -1661,7 +1661,7 @@
       <c r="E15" s="2" t="n"/>
       <c r="F15" s="2" t="n"/>
       <c r="G15" s="10">
-        <f>IF($F15="","",AND(IF($B15="",TRUE,VLOOKUP($B15,Faits!$A:$B,2,FALSE)),IF($C15="",TRUE,VLOOKUP($C15,Faits!$A:$B,2,FALSE)),IF($D15="",TRUE,VLOOKUP($D15,Faits!$A:$B,2,FALSE)),IF($E15="",TRUE,VLOOKUP($E15,Faits!$A:$B,2,FALSE)),NOT(VLOOKUP($F15,Faits!$A:$B,2,FALSE))))</f>
+        <f>IF($F15="","",AND(IF($B15="",TRUE,VLOOKUP($B15,Faits!$A:$B,2,FALSE)=TRUE),IF($C15="",TRUE,VLOOKUP($C15,Faits!$A:$B,2,FALSE)=TRUE),IF($D15="",TRUE,VLOOKUP($D15,Faits!$A:$B,2,FALSE)=TRUE),IF($E15="",TRUE,VLOOKUP($E15,Faits!$A:$B,2,FALSE)=TRUE),VLOOKUP($F15,Faits!$A:$B,2,FALSE)&lt;&gt;TRUE))</f>
         <v/>
       </c>
       <c r="H15" s="10">
@@ -1677,7 +1677,7 @@
       <c r="E16" s="2" t="n"/>
       <c r="F16" s="2" t="n"/>
       <c r="G16" s="10">
-        <f>IF($F16="","",AND(IF($B16="",TRUE,VLOOKUP($B16,Faits!$A:$B,2,FALSE)),IF($C16="",TRUE,VLOOKUP($C16,Faits!$A:$B,2,FALSE)),IF($D16="",TRUE,VLOOKUP($D16,Faits!$A:$B,2,FALSE)),IF($E16="",TRUE,VLOOKUP($E16,Faits!$A:$B,2,FALSE)),NOT(VLOOKUP($F16,Faits!$A:$B,2,FALSE))))</f>
+        <f>IF($F16="","",AND(IF($B16="",TRUE,VLOOKUP($B16,Faits!$A:$B,2,FALSE)=TRUE),IF($C16="",TRUE,VLOOKUP($C16,Faits!$A:$B,2,FALSE)=TRUE),IF($D16="",TRUE,VLOOKUP($D16,Faits!$A:$B,2,FALSE)=TRUE),IF($E16="",TRUE,VLOOKUP($E16,Faits!$A:$B,2,FALSE)=TRUE),VLOOKUP($F16,Faits!$A:$B,2,FALSE)&lt;&gt;TRUE))</f>
         <v/>
       </c>
       <c r="H16" s="10">
@@ -1693,7 +1693,7 @@
       <c r="E17" s="2" t="n"/>
       <c r="F17" s="2" t="n"/>
       <c r="G17" s="10">
-        <f>IF($F17="","",AND(IF($B17="",TRUE,VLOOKUP($B17,Faits!$A:$B,2,FALSE)),IF($C17="",TRUE,VLOOKUP($C17,Faits!$A:$B,2,FALSE)),IF($D17="",TRUE,VLOOKUP($D17,Faits!$A:$B,2,FALSE)),IF($E17="",TRUE,VLOOKUP($E17,Faits!$A:$B,2,FALSE)),NOT(VLOOKUP($F17,Faits!$A:$B,2,FALSE))))</f>
+        <f>IF($F17="","",AND(IF($B17="",TRUE,VLOOKUP($B17,Faits!$A:$B,2,FALSE)=TRUE),IF($C17="",TRUE,VLOOKUP($C17,Faits!$A:$B,2,FALSE)=TRUE),IF($D17="",TRUE,VLOOKUP($D17,Faits!$A:$B,2,FALSE)=TRUE),IF($E17="",TRUE,VLOOKUP($E17,Faits!$A:$B,2,FALSE)=TRUE),VLOOKUP($F17,Faits!$A:$B,2,FALSE)&lt;&gt;TRUE))</f>
         <v/>
       </c>
       <c r="H17" s="10">
@@ -1709,7 +1709,7 @@
       <c r="E18" s="2" t="n"/>
       <c r="F18" s="2" t="n"/>
       <c r="G18" s="10">
-        <f>IF($F18="","",AND(IF($B18="",TRUE,VLOOKUP($B18,Faits!$A:$B,2,FALSE)),IF($C18="",TRUE,VLOOKUP($C18,Faits!$A:$B,2,FALSE)),IF($D18="",TRUE,VLOOKUP($D18,Faits!$A:$B,2,FALSE)),IF($E18="",TRUE,VLOOKUP($E18,Faits!$A:$B,2,FALSE)),NOT(VLOOKUP($F18,Faits!$A:$B,2,FALSE))))</f>
+        <f>IF($F18="","",AND(IF($B18="",TRUE,VLOOKUP($B18,Faits!$A:$B,2,FALSE)=TRUE),IF($C18="",TRUE,VLOOKUP($C18,Faits!$A:$B,2,FALSE)=TRUE),IF($D18="",TRUE,VLOOKUP($D18,Faits!$A:$B,2,FALSE)=TRUE),IF($E18="",TRUE,VLOOKUP($E18,Faits!$A:$B,2,FALSE)=TRUE),VLOOKUP($F18,Faits!$A:$B,2,FALSE)&lt;&gt;TRUE))</f>
         <v/>
       </c>
       <c r="H18" s="10">
@@ -1725,7 +1725,7 @@
       <c r="E19" s="2" t="n"/>
       <c r="F19" s="2" t="n"/>
       <c r="G19" s="10">
-        <f>IF($F19="","",AND(IF($B19="",TRUE,VLOOKUP($B19,Faits!$A:$B,2,FALSE)),IF($C19="",TRUE,VLOOKUP($C19,Faits!$A:$B,2,FALSE)),IF($D19="",TRUE,VLOOKUP($D19,Faits!$A:$B,2,FALSE)),IF($E19="",TRUE,VLOOKUP($E19,Faits!$A:$B,2,FALSE)),NOT(VLOOKUP($F19,Faits!$A:$B,2,FALSE))))</f>
+        <f>IF($F19="","",AND(IF($B19="",TRUE,VLOOKUP($B19,Faits!$A:$B,2,FALSE)=TRUE),IF($C19="",TRUE,VLOOKUP($C19,Faits!$A:$B,2,FALSE)=TRUE),IF($D19="",TRUE,VLOOKUP($D19,Faits!$A:$B,2,FALSE)=TRUE),IF($E19="",TRUE,VLOOKUP($E19,Faits!$A:$B,2,FALSE)=TRUE),VLOOKUP($F19,Faits!$A:$B,2,FALSE)&lt;&gt;TRUE))</f>
         <v/>
       </c>
       <c r="H19" s="10">
@@ -1741,7 +1741,7 @@
       <c r="E20" s="2" t="n"/>
       <c r="F20" s="2" t="n"/>
       <c r="G20" s="10">
-        <f>IF($F20="","",AND(IF($B20="",TRUE,VLOOKUP($B20,Faits!$A:$B,2,FALSE)),IF($C20="",TRUE,VLOOKUP($C20,Faits!$A:$B,2,FALSE)),IF($D20="",TRUE,VLOOKUP($D20,Faits!$A:$B,2,FALSE)),IF($E20="",TRUE,VLOOKUP($E20,Faits!$A:$B,2,FALSE)),NOT(VLOOKUP($F20,Faits!$A:$B,2,FALSE))))</f>
+        <f>IF($F20="","",AND(IF($B20="",TRUE,VLOOKUP($B20,Faits!$A:$B,2,FALSE)=TRUE),IF($C20="",TRUE,VLOOKUP($C20,Faits!$A:$B,2,FALSE)=TRUE),IF($D20="",TRUE,VLOOKUP($D20,Faits!$A:$B,2,FALSE)=TRUE),IF($E20="",TRUE,VLOOKUP($E20,Faits!$A:$B,2,FALSE)=TRUE),VLOOKUP($F20,Faits!$A:$B,2,FALSE)&lt;&gt;TRUE))</f>
         <v/>
       </c>
       <c r="H20" s="10">
@@ -1757,7 +1757,7 @@
       <c r="E21" s="2" t="n"/>
       <c r="F21" s="2" t="n"/>
       <c r="G21" s="10">
-        <f>IF($F21="","",AND(IF($B21="",TRUE,VLOOKUP($B21,Faits!$A:$B,2,FALSE)),IF($C21="",TRUE,VLOOKUP($C21,Faits!$A:$B,2,FALSE)),IF($D21="",TRUE,VLOOKUP($D21,Faits!$A:$B,2,FALSE)),IF($E21="",TRUE,VLOOKUP($E21,Faits!$A:$B,2,FALSE)),NOT(VLOOKUP($F21,Faits!$A:$B,2,FALSE))))</f>
+        <f>IF($F21="","",AND(IF($B21="",TRUE,VLOOKUP($B21,Faits!$A:$B,2,FALSE)=TRUE),IF($C21="",TRUE,VLOOKUP($C21,Faits!$A:$B,2,FALSE)=TRUE),IF($D21="",TRUE,VLOOKUP($D21,Faits!$A:$B,2,FALSE)=TRUE),IF($E21="",TRUE,VLOOKUP($E21,Faits!$A:$B,2,FALSE)=TRUE),VLOOKUP($F21,Faits!$A:$B,2,FALSE)&lt;&gt;TRUE))</f>
         <v/>
       </c>
       <c r="H21" s="10">
@@ -1773,7 +1773,7 @@
       <c r="E22" s="2" t="n"/>
       <c r="F22" s="2" t="n"/>
       <c r="G22" s="10">
-        <f>IF($F22="","",AND(IF($B22="",TRUE,VLOOKUP($B22,Faits!$A:$B,2,FALSE)),IF($C22="",TRUE,VLOOKUP($C22,Faits!$A:$B,2,FALSE)),IF($D22="",TRUE,VLOOKUP($D22,Faits!$A:$B,2,FALSE)),IF($E22="",TRUE,VLOOKUP($E22,Faits!$A:$B,2,FALSE)),NOT(VLOOKUP($F22,Faits!$A:$B,2,FALSE))))</f>
+        <f>IF($F22="","",AND(IF($B22="",TRUE,VLOOKUP($B22,Faits!$A:$B,2,FALSE)=TRUE),IF($C22="",TRUE,VLOOKUP($C22,Faits!$A:$B,2,FALSE)=TRUE),IF($D22="",TRUE,VLOOKUP($D22,Faits!$A:$B,2,FALSE)=TRUE),IF($E22="",TRUE,VLOOKUP($E22,Faits!$A:$B,2,FALSE)=TRUE),VLOOKUP($F22,Faits!$A:$B,2,FALSE)&lt;&gt;TRUE))</f>
         <v/>
       </c>
       <c r="H22" s="10">

</xml_diff>